<commit_message>
added ABCD-label switch, added shortkeys for revealing answers
</commit_message>
<xml_diff>
--- a/Der_Große_Preis_Template.xlsx
+++ b/Der_Große_Preis_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Max\Documents\Ferienlager\Der Große Preis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Max\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23314CF9-F7D3-40D8-A513-7B634FA56908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C90BF5-E466-4F80-8759-1C9BBCC77EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2985" yWindow="2985" windowWidth="24105" windowHeight="11955" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="der_grosse_preis" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="19">
   <si>
     <t>Kategorien</t>
   </si>
@@ -93,7 +93,13 @@
     <t>Frage mit vier Antwortmöglichkeiten?</t>
   </si>
   <si>
-    <t>falsche Antwort</t>
+    <t>falsche Antwort 1</t>
+  </si>
+  <si>
+    <t>falsche Antwort 2</t>
+  </si>
+  <si>
+    <t>falsche Antwort 3</t>
   </si>
 </sst>
 </file>
@@ -586,7 +592,7 @@
       <c r="AB1" s="1"/>
       <c r="AC1" s="1"/>
     </row>
-    <row r="2" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>7</v>
       </c>
@@ -628,7 +634,7 @@
       <c r="AB2" s="1"/>
       <c r="AC2" s="1"/>
     </row>
-    <row r="3" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>8</v>
       </c>
@@ -650,10 +656,10 @@
         <v>16</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -676,7 +682,7 @@
       <c r="AB3" s="1"/>
       <c r="AC3" s="1"/>
     </row>
-    <row r="4" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>9</v>
       </c>
@@ -694,14 +700,14 @@
       <c r="F4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="13">
-        <v>0.02</v>
+      <c r="G4" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H4" s="6">
-        <v>0.03</v>
+      <c r="H4" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I4" s="7">
-        <v>0.04</v>
+      <c r="I4" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -724,7 +730,7 @@
       <c r="AB4" s="1"/>
       <c r="AC4" s="1"/>
     </row>
-    <row r="5" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>10</v>
       </c>
@@ -742,14 +748,14 @@
       <c r="F5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="13">
-        <v>0.02</v>
+      <c r="G5" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H5" s="6">
-        <v>0.03</v>
+      <c r="H5" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I5" s="7">
-        <v>0.04</v>
+      <c r="I5" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -772,7 +778,7 @@
       <c r="AB5" s="1"/>
       <c r="AC5" s="1"/>
     </row>
-    <row r="6" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>11</v>
       </c>
@@ -790,14 +796,14 @@
       <c r="F6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="13">
-        <v>0.02</v>
+      <c r="G6" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H6" s="6">
-        <v>0.03</v>
+      <c r="H6" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I6" s="7">
-        <v>0.04</v>
+      <c r="I6" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
@@ -820,7 +826,7 @@
       <c r="AB6" s="1"/>
       <c r="AC6" s="1"/>
     </row>
-    <row r="7" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>12</v>
       </c>
@@ -836,14 +842,14 @@
       <c r="F7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="13">
-        <v>0.02</v>
+      <c r="G7" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H7" s="6">
-        <v>0.03</v>
+      <c r="H7" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I7" s="7">
-        <v>0.04</v>
+      <c r="I7" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -866,7 +872,7 @@
       <c r="AB7" s="1"/>
       <c r="AC7" s="1"/>
     </row>
-    <row r="8" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -880,14 +886,14 @@
       <c r="F8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="13">
-        <v>0.02</v>
+      <c r="G8" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H8" s="6">
-        <v>0.03</v>
+      <c r="H8" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I8" s="7">
-        <v>0.04</v>
+      <c r="I8" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -910,7 +916,7 @@
       <c r="AB8" s="1"/>
       <c r="AC8" s="1"/>
     </row>
-    <row r="9" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -924,14 +930,14 @@
       <c r="F9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="13">
-        <v>0.02</v>
+      <c r="G9" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H9" s="6">
-        <v>0.03</v>
+      <c r="H9" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I9" s="7">
-        <v>0.04</v>
+      <c r="I9" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
@@ -954,7 +960,7 @@
       <c r="AB9" s="1"/>
       <c r="AC9" s="1"/>
     </row>
-    <row r="10" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -968,14 +974,14 @@
       <c r="F10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="13">
-        <v>0.02</v>
+      <c r="G10" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H10" s="6">
-        <v>0.03</v>
+      <c r="H10" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I10" s="7">
-        <v>0.04</v>
+      <c r="I10" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
@@ -998,7 +1004,7 @@
       <c r="AB10" s="1"/>
       <c r="AC10" s="1"/>
     </row>
-    <row r="11" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -1012,14 +1018,14 @@
       <c r="F11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="13">
-        <v>0.02</v>
+      <c r="G11" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H11" s="6">
-        <v>0.03</v>
+      <c r="H11" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I11" s="7">
-        <v>0.04</v>
+      <c r="I11" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
@@ -1042,7 +1048,7 @@
       <c r="AB11" s="1"/>
       <c r="AC11" s="1"/>
     </row>
-    <row r="12" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1056,14 +1062,14 @@
       <c r="F12" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="13">
-        <v>0.02</v>
+      <c r="G12" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H12" s="6">
-        <v>0.03</v>
+      <c r="H12" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I12" s="7">
-        <v>0.04</v>
+      <c r="I12" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
@@ -1086,7 +1092,7 @@
       <c r="AB12" s="1"/>
       <c r="AC12" s="1"/>
     </row>
-    <row r="13" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1100,14 +1106,14 @@
       <c r="F13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="13">
-        <v>0.02</v>
+      <c r="G13" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H13" s="6">
-        <v>0.03</v>
+      <c r="H13" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I13" s="7">
-        <v>0.04</v>
+      <c r="I13" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
@@ -1130,7 +1136,7 @@
       <c r="AB13" s="1"/>
       <c r="AC13" s="1"/>
     </row>
-    <row r="14" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -1144,14 +1150,14 @@
       <c r="F14" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G14" s="13">
-        <v>0.02</v>
+      <c r="G14" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H14" s="6">
-        <v>0.03</v>
+      <c r="H14" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I14" s="7">
-        <v>0.04</v>
+      <c r="I14" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
@@ -1174,7 +1180,7 @@
       <c r="AB14" s="1"/>
       <c r="AC14" s="1"/>
     </row>
-    <row r="15" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -1188,14 +1194,14 @@
       <c r="F15" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G15" s="13">
-        <v>0.02</v>
+      <c r="G15" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H15" s="6">
-        <v>0.03</v>
+      <c r="H15" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I15" s="7">
-        <v>0.04</v>
+      <c r="I15" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
@@ -1218,7 +1224,7 @@
       <c r="AB15" s="1"/>
       <c r="AC15" s="1"/>
     </row>
-    <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
@@ -1232,14 +1238,14 @@
       <c r="F16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G16" s="13">
-        <v>0.02</v>
+      <c r="G16" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H16" s="6">
-        <v>0.03</v>
+      <c r="H16" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I16" s="7">
-        <v>0.04</v>
+      <c r="I16" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -1262,7 +1268,7 @@
       <c r="AB16" s="1"/>
       <c r="AC16" s="1"/>
     </row>
-    <row r="17" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -1276,14 +1282,14 @@
       <c r="F17" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G17" s="13">
-        <v>0.02</v>
+      <c r="G17" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H17" s="6">
-        <v>0.03</v>
+      <c r="H17" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I17" s="7">
-        <v>0.04</v>
+      <c r="I17" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -1306,7 +1312,7 @@
       <c r="AB17" s="1"/>
       <c r="AC17" s="1"/>
     </row>
-    <row r="18" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -1320,14 +1326,14 @@
       <c r="F18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G18" s="13">
-        <v>0.02</v>
+      <c r="G18" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H18" s="6">
-        <v>0.03</v>
+      <c r="H18" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I18" s="7">
-        <v>0.04</v>
+      <c r="I18" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -1350,7 +1356,7 @@
       <c r="AB18" s="1"/>
       <c r="AC18" s="1"/>
     </row>
-    <row r="19" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -1364,14 +1370,14 @@
       <c r="F19" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G19" s="13">
-        <v>0.02</v>
+      <c r="G19" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H19" s="6">
-        <v>0.03</v>
+      <c r="H19" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I19" s="7">
-        <v>0.04</v>
+      <c r="I19" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
@@ -1394,7 +1400,7 @@
       <c r="AB19" s="1"/>
       <c r="AC19" s="1"/>
     </row>
-    <row r="20" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
@@ -1408,14 +1414,14 @@
       <c r="F20" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G20" s="13">
-        <v>0.02</v>
+      <c r="G20" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H20" s="6">
-        <v>0.03</v>
+      <c r="H20" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I20" s="7">
-        <v>0.04</v>
+      <c r="I20" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
@@ -1438,7 +1444,7 @@
       <c r="AB20" s="1"/>
       <c r="AC20" s="1"/>
     </row>
-    <row r="21" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
@@ -1452,14 +1458,14 @@
       <c r="F21" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G21" s="13">
-        <v>0.02</v>
+      <c r="G21" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H21" s="6">
-        <v>0.03</v>
+      <c r="H21" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I21" s="7">
-        <v>0.04</v>
+      <c r="I21" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
@@ -1482,7 +1488,7 @@
       <c r="AB21" s="1"/>
       <c r="AC21" s="1"/>
     </row>
-    <row r="22" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1496,14 +1502,14 @@
       <c r="F22" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G22" s="13">
-        <v>0.02</v>
+      <c r="G22" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H22" s="6">
-        <v>0.03</v>
+      <c r="H22" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I22" s="7">
-        <v>0.04</v>
+      <c r="I22" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
@@ -1526,7 +1532,7 @@
       <c r="AB22" s="1"/>
       <c r="AC22" s="1"/>
     </row>
-    <row r="23" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1540,14 +1546,14 @@
       <c r="F23" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G23" s="13">
-        <v>0.02</v>
+      <c r="G23" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H23" s="6">
-        <v>0.03</v>
+      <c r="H23" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I23" s="7">
-        <v>0.04</v>
+      <c r="I23" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
@@ -1570,7 +1576,7 @@
       <c r="AB23" s="1"/>
       <c r="AC23" s="1"/>
     </row>
-    <row r="24" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
@@ -1584,14 +1590,14 @@
       <c r="F24" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G24" s="13">
-        <v>0.02</v>
+      <c r="G24" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H24" s="6">
-        <v>0.03</v>
+      <c r="H24" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I24" s="7">
-        <v>0.04</v>
+      <c r="I24" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
@@ -1614,7 +1620,7 @@
       <c r="AB24" s="1"/>
       <c r="AC24" s="1"/>
     </row>
-    <row r="25" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
@@ -1628,14 +1634,14 @@
       <c r="F25" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G25" s="13">
-        <v>0.02</v>
+      <c r="G25" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H25" s="6">
-        <v>0.03</v>
+      <c r="H25" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I25" s="7">
-        <v>0.04</v>
+      <c r="I25" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
@@ -1658,7 +1664,7 @@
       <c r="AB25" s="1"/>
       <c r="AC25" s="1"/>
     </row>
-    <row r="26" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
@@ -1672,14 +1678,14 @@
       <c r="F26" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G26" s="13">
-        <v>0.02</v>
+      <c r="G26" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H26" s="6">
-        <v>0.03</v>
+      <c r="H26" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I26" s="7">
-        <v>0.04</v>
+      <c r="I26" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
@@ -1702,7 +1708,7 @@
       <c r="AB26" s="1"/>
       <c r="AC26" s="1"/>
     </row>
-    <row r="27" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -1716,14 +1722,14 @@
       <c r="F27" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G27" s="13">
-        <v>0.02</v>
+      <c r="G27" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H27" s="6">
-        <v>0.03</v>
+      <c r="H27" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I27" s="7">
-        <v>0.04</v>
+      <c r="I27" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
@@ -1746,7 +1752,7 @@
       <c r="AB27" s="1"/>
       <c r="AC27" s="1"/>
     </row>
-    <row r="28" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -1760,14 +1766,14 @@
       <c r="F28" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G28" s="13">
-        <v>0.02</v>
+      <c r="G28" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H28" s="6">
-        <v>0.03</v>
+      <c r="H28" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I28" s="7">
-        <v>0.04</v>
+      <c r="I28" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
@@ -1790,7 +1796,7 @@
       <c r="AB28" s="1"/>
       <c r="AC28" s="1"/>
     </row>
-    <row r="29" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -1804,14 +1810,14 @@
       <c r="F29" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G29" s="13">
-        <v>0.02</v>
+      <c r="G29" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H29" s="6">
-        <v>0.03</v>
+      <c r="H29" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I29" s="7">
-        <v>0.04</v>
+      <c r="I29" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
@@ -1834,7 +1840,7 @@
       <c r="AB29" s="1"/>
       <c r="AC29" s="1"/>
     </row>
-    <row r="30" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1848,14 +1854,14 @@
       <c r="F30" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G30" s="13">
-        <v>0.02</v>
+      <c r="G30" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H30" s="6">
-        <v>0.03</v>
+      <c r="H30" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I30" s="7">
-        <v>0.04</v>
+      <c r="I30" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
@@ -1878,7 +1884,7 @@
       <c r="AB30" s="1"/>
       <c r="AC30" s="1"/>
     </row>
-    <row r="31" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:29" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -1892,14 +1898,14 @@
       <c r="F31" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G31" s="13">
-        <v>0.02</v>
+      <c r="G31" s="13" t="s">
+        <v>16</v>
       </c>
-      <c r="H31" s="6">
-        <v>0.03</v>
+      <c r="H31" s="6" t="s">
+        <v>17</v>
       </c>
-      <c r="I31" s="7">
-        <v>0.04</v>
+      <c r="I31" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>

</xml_diff>